<commit_message>
Update Lesson 02 Excel Analysis
</commit_message>
<xml_diff>
--- a/Lesson-02/Sales_Tables.xlsx
+++ b/Lesson-02/Sales_Tables.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4247A7D5-F155-42CE-A648-6A39271EC6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{D878CB2A-0C84-4ED9-AF96-21610F407CA2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{D878CB2A-0C84-4ED9-AF96-21610F407CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="RawData" sheetId="1" r:id="rId1"/>
@@ -350,12 +350,12 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C09B3307-CC35-41D3-BAFE-A8B7854D4BB2}" name="Date" totalsRowLabel="Total" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{C09B3307-CC35-41D3-BAFE-A8B7854D4BB2}" name="Date" totalsRowLabel="Total" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{A85C4C07-5DC0-4F19-9C89-423F52B2366F}" name="Product"/>
     <tableColumn id="3" xr3:uid="{F04F31EE-8069-4115-A47F-CF5155EB9972}" name="Category"/>
     <tableColumn id="4" xr3:uid="{45439CD0-6471-4E45-B1A0-0CCFF58558DE}" name="Quantity"/>
     <tableColumn id="5" xr3:uid="{2576F4B3-C800-4206-853E-6910080DE689}" name="Unit Price"/>
-    <tableColumn id="6" xr3:uid="{494A7127-D9BF-452D-96B3-2C346E3F5497}" name="Revenue" totalsRowFunction="sum" dataDxfId="5">
+    <tableColumn id="6" xr3:uid="{494A7127-D9BF-452D-96B3-2C346E3F5497}" name="Revenue" totalsRowFunction="sum" dataDxfId="0">
       <calculatedColumnFormula>Table5[[#This Row],[Quantity]]*Table5[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -367,12 +367,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E4FA6493-19ED-4DDA-B2EA-E39D8F8EBFED}" name="FinalTable" displayName="FinalTable" ref="A1:F102" totalsRowCount="1">
   <autoFilter ref="A1:F101" xr:uid="{E4FA6493-19ED-4DDA-B2EA-E39D8F8EBFED}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{72517A94-5138-466B-AC92-A44AB23DD454}" name="Date" totalsRowLabel="Total" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{72517A94-5138-466B-AC92-A44AB23DD454}" name="Date" totalsRowLabel="Total" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{93A2BF68-44E2-46D9-A484-2CABEF6FD221}" name="Product"/>
     <tableColumn id="3" xr3:uid="{D44C6A7B-F3E4-4F2F-ACF4-2A7C8E5D6312}" name="Category"/>
     <tableColumn id="4" xr3:uid="{C9BE252A-EEFC-4B28-A61B-0677FDE1540D}" name="Quantity"/>
     <tableColumn id="5" xr3:uid="{FDEE569B-A3B2-45AE-A7D5-9BDD44E6F604}" name="Unit Price"/>
-    <tableColumn id="6" xr3:uid="{CC24B8CB-8B58-4711-9409-9A100363F02C}" name="Revenue" totalsRowFunction="sum" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{CC24B8CB-8B58-4711-9409-9A100363F02C}" name="Revenue" totalsRowFunction="sum" dataDxfId="5">
       <calculatedColumnFormula>FinalTable[[#This Row],[Quantity]]*FinalTable[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>

<commit_message>
Update sales analysis workbook
</commit_message>
<xml_diff>
--- a/Lesson-02/Sales_Tables.xlsx
+++ b/Lesson-02/Sales_Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Excel_Data_Analyst_Journey\Lesson-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4247A7D5-F155-42CE-A648-6A39271EC6C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF02EAE-F678-461B-9D1F-7DEE1482B062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{D878CB2A-0C84-4ED9-AF96-21610F407CA2}"/>
+    <workbookView minimized="1" xWindow="3210" yWindow="1080" windowWidth="15375" windowHeight="7875" activeTab="1" xr2:uid="{D878CB2A-0C84-4ED9-AF96-21610F407CA2}"/>
   </bookViews>
   <sheets>
     <sheet name="RawData" sheetId="1" r:id="rId1"/>
@@ -327,12 +327,12 @@
     <sortCondition descending="1" ref="G2:G102"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{98389B45-1E01-4FC3-836E-9D779C4A27C9}" name="Date" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{98389B45-1E01-4FC3-836E-9D779C4A27C9}" name="Date" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{7605C53F-3AC4-41DB-A5AC-4DCF3DD5154C}" name="Product"/>
     <tableColumn id="3" xr3:uid="{E696BC51-E797-4CBB-804C-2C70D0C9DC1E}" name="Category"/>
     <tableColumn id="4" xr3:uid="{02F2FBB5-A448-49F4-B0ED-B620B864E872}" name="Quantity"/>
     <tableColumn id="5" xr3:uid="{391693B0-95E7-45BD-A9C2-F1EEB2E67B39}" name="Unit Price"/>
-    <tableColumn id="7" xr3:uid="{B58ABED8-C09E-43CB-B152-F00716392A11}" name="Revenue" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{B58ABED8-C09E-43CB-B152-F00716392A11}" name="Revenue" dataDxfId="5">
       <calculatedColumnFormula>Table2[[#This Row],[Quantity]]*Table2[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -350,12 +350,12 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C09B3307-CC35-41D3-BAFE-A8B7854D4BB2}" name="Date" totalsRowLabel="Total" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C09B3307-CC35-41D3-BAFE-A8B7854D4BB2}" name="Date" totalsRowLabel="Total" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{A85C4C07-5DC0-4F19-9C89-423F52B2366F}" name="Product"/>
     <tableColumn id="3" xr3:uid="{F04F31EE-8069-4115-A47F-CF5155EB9972}" name="Category"/>
     <tableColumn id="4" xr3:uid="{45439CD0-6471-4E45-B1A0-0CCFF58558DE}" name="Quantity"/>
     <tableColumn id="5" xr3:uid="{2576F4B3-C800-4206-853E-6910080DE689}" name="Unit Price"/>
-    <tableColumn id="6" xr3:uid="{494A7127-D9BF-452D-96B3-2C346E3F5497}" name="Revenue" totalsRowFunction="sum" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{494A7127-D9BF-452D-96B3-2C346E3F5497}" name="Revenue" totalsRowFunction="sum" dataDxfId="2">
       <calculatedColumnFormula>Table5[[#This Row],[Quantity]]*Table5[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -367,12 +367,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E4FA6493-19ED-4DDA-B2EA-E39D8F8EBFED}" name="FinalTable" displayName="FinalTable" ref="A1:F102" totalsRowCount="1">
   <autoFilter ref="A1:F101" xr:uid="{E4FA6493-19ED-4DDA-B2EA-E39D8F8EBFED}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{72517A94-5138-466B-AC92-A44AB23DD454}" name="Date" totalsRowLabel="Total" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{72517A94-5138-466B-AC92-A44AB23DD454}" name="Date" totalsRowLabel="Total" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{93A2BF68-44E2-46D9-A484-2CABEF6FD221}" name="Product"/>
     <tableColumn id="3" xr3:uid="{D44C6A7B-F3E4-4F2F-ACF4-2A7C8E5D6312}" name="Category"/>
     <tableColumn id="4" xr3:uid="{C9BE252A-EEFC-4B28-A61B-0677FDE1540D}" name="Quantity"/>
     <tableColumn id="5" xr3:uid="{FDEE569B-A3B2-45AE-A7D5-9BDD44E6F604}" name="Unit Price"/>
-    <tableColumn id="6" xr3:uid="{CC24B8CB-8B58-4711-9409-9A100363F02C}" name="Revenue" totalsRowFunction="sum" dataDxfId="5">
+    <tableColumn id="6" xr3:uid="{CC24B8CB-8B58-4711-9409-9A100363F02C}" name="Revenue" totalsRowFunction="sum" dataDxfId="0">
       <calculatedColumnFormula>FinalTable[[#This Row],[Quantity]]*FinalTable[[#This Row],[Unit Price]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>